<commit_message>
Update soccer trades 2026-08-16 16:03:16 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/English Premier League/trades.xlsx
+++ b/data/sxbet/ligas/English Premier League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x7d536b1f35b725269abc7254ec90ca50ccca56bb210b3d2118963062a41ce0b2</t>
+          <t>0x68b08a65cfbca371bd6e5fb708f67ec87d89cc9bbce85a8e7713f418d841b56e</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>39.22095</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.4825</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>English Premier League</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Hull City vs Manchester United</t>
+          <t>Brentford vs Tottenham Hotspur</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Hull City</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Manchester United</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x2cf719d8125a0ce8b30cf64e54c5ecf77f06126bc554e7b25fabbc72ee413952</t>
+          <t>0x5745247ce80bf8689dfe06022d99547fa927b160a694591736f58a9fb1d8b0b3</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19236539</t>
+          <t>L19236538</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786884152</t>
+          <t>1786893348</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1787398200</t>
+          <t>1787416200</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>124.510952</t>
+          <t>10.362694</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,31 +635,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x3b4020a7dedef04108fd84d51b986ec0aa64b0e777c9ac0d4c51f107d3590106</t>
+          <t>0xdccedeb81191ae5ca0020d7b88a47d494efefcd5d43bb52471ac8a338b980d63</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6.47</t>
+          <t>83.27998</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.2138</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>English Premier League</t>
@@ -667,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Hull City vs Manchester United</t>
+          <t>Brentford vs Tottenham Hotspur</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Hull City</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Manchester United</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xff94b64540b1f4876a9b61f7abc856bf1efeb99bca7cf7fc56e51fbe432c69a3</t>
+          <t>0xe5b7688e1a022a4e8890c76b076baf5a197eb6a99074e068e78cf90d235575f1</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19236539</t>
+          <t>L19236538</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -712,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786880633</t>
+          <t>1786893337</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1787398200</t>
+          <t>1787416200</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>30.269006</t>
+          <t>112.350732</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xe4c2b9f486982b41626561d2f921b54a2cc40bdf036a0442449bf08b0d587a84</t>
+          <t>0x392d16c666fb526b77db1e14f2769e23b06ec209badf92ce737f19734622203d</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -747,23 +755,31 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>123.26515</t>
+          <t>109.09</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5787</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>English Premier League</t>
@@ -771,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Hull City vs Manchester United</t>
+          <t>Brentford vs Tottenham Hotspur</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Hull City</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Manchester United</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xfa50abbae5bfdbf97cd2a58fbf350d5eba025159d6ca11f20066807fbf6cfcd2</t>
+          <t>0xca0eca2f3775c1a08e62703b0bc5096c0190a2a3e31600680143794ea7df898c</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19236539</t>
+          <t>L19236538</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -816,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786880266</t>
+          <t>1786893337</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1787398200</t>
+          <t>1787416200</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>212.98514</t>
+          <t>311.685714</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,102 +859,854 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>0xd0bd4ac629ca0911ce51fad27d2f6e4e238bbaa1d989cbe664817ee4ebfcb2fc</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>75.19</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.2175</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Brentford vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xa0f6617255819010f00be4fb75d4597b30a12ae0fb712dd0c531651c52923088</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19236538</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1786893336</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1787416200</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>345.701149</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0x869c335bdd3d2636e2f37a4d6ae91ebd65feaf4d359d1dbc8a5638d0d44406d8</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>283.08</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.5375</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Brentford 0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Brentford vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x116f827edbab2c40b76f0d489ef752efa0705d0d7281eb667522cfc3e453d283</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19236538</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1786893336</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1787416200</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>526.660465</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0x33233046e450a9042a0668b9a365ed1860e6833e33da55a35b5c6466d4648203</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>29.60265</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.4825</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Brentford vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0x5745247ce80bf8689dfe06022d99547fa927b160a694591736f58a9fb1d8b0b3</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19236538</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1786893336</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1787416200</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>61.352642</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0x28b4cf2ef0b8471323b75e91b77f80e7f227ce9488635fc5dd9e23671ba1dcd4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>221.34</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Brentford vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x3212fdea7fa0e385d3d02eb680e1ce50a1c7cb58afa9e7e34eb266a06ab18871</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19236538</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1786893336</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1787416200</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>491.866667</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0x7d536b1f35b725269abc7254ec90ca50ccca56bb210b3d2118963062a41ce0b2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>39.22095</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.315</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Hull City vs Manchester United</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0x2cf719d8125a0ce8b30cf64e54c5ecf77f06126bc554e7b25fabbc72ee413952</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19236539</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1786884152</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1787398200</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>124.510952</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0x3b4020a7dedef04108fd84d51b986ec0aa64b0e777c9ac0d4c51f107d3590106</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>6.47</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.2138</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Hull City vs Manchester United</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0xff94b64540b1f4876a9b61f7abc856bf1efeb99bca7cf7fc56e51fbe432c69a3</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19236539</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786880633</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1787398200</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>30.269006</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0xe4c2b9f486982b41626561d2f921b54a2cc40bdf036a0442449bf08b0d587a84</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>123.26515</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.5787</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Hull City vs Manchester United</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0xfa50abbae5bfdbf97cd2a58fbf350d5eba025159d6ca11f20066807fbf6cfcd2</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19236539</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786880266</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1787398200</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>212.98514</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>0x0353c141478d0566f83e374f7784af6eb93f5721a343bd2253347a401c09996e</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
         <is>
           <t>60.54972</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>1.6738</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Under/Over (3.5)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
         <is>
           <t>English Premier League</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Hull City vs Manchester United</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Hull City</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Manchester United</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>0x0a08e0170f01c3d1a9a1ac32f64197e2b46643bdbadcccc75996936c0470d731</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>L19236539</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>1786880265</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>1787398200</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>89.869714</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-16 18:03:12 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/English Premier League/trades.xlsx
+++ b/data/sxbet/ligas/English Premier League/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x68b08a65cfbca371bd6e5fb708f67ec87d89cc9bbce85a8e7713f418d841b56e</t>
+          <t>0x8972a038094c2b563424c3acec352962380c3b7e5e39c3f0a4c41fbe6bb72bd7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>207.22</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4825</t>
+          <t>1.4338</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>English Premier League</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x5745247ce80bf8689dfe06022d99547fa927b160a694591736f58a9fb1d8b0b3</t>
+          <t>0x0a314280e77d81763d7ca8768681a92b211153ea82e8cc52f29060bc6d5e30fe</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786893348</t>
+          <t>1786902966</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>10.362694</t>
+          <t>477.740634</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,92 +635,84 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xdccedeb81191ae5ca0020d7b88a47d494efefcd5d43bb52471ac8a338b980d63</t>
+          <t>0x68b08a65cfbca371bd6e5fb708f67ec87d89cc9bbce85a8e7713f418d841b56e</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+          <t>0x0DeAbC808957aBc9f4778C03b03CC1D2cBBC9D60</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.4825</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Brentford vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x5745247ce80bf8689dfe06022d99547fa927b160a694591736f58a9fb1d8b0b3</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19236538</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>83.27998</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1.7412</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>English Premier League</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Brentford vs Tottenham Hotspur</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Brentford</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Tottenham Hotspur</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0xe5b7688e1a022a4e8890c76b076baf5a197eb6a99074e068e78cf90d235575f1</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>L19236538</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786893337</t>
+          <t>1786893348</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>112.350732</t>
+          <t>10.362694</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +739,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x392d16c666fb526b77db1e14f2769e23b06ec209badf92ce737f19734622203d</t>
+          <t>0xdccedeb81191ae5ca0020d7b88a47d494efefcd5d43bb52471ac8a338b980d63</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -762,22 +754,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>109.09</t>
+          <t>83.27998</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -802,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xca0eca2f3775c1a08e62703b0bc5096c0190a2a3e31600680143794ea7df898c</t>
+          <t>0xe5b7688e1a022a4e8890c76b076baf5a197eb6a99074e068e78cf90d235575f1</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -842,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>311.685714</t>
+          <t>112.350732</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xd0bd4ac629ca0911ce51fad27d2f6e4e238bbaa1d989cbe664817ee4ebfcb2fc</t>
+          <t>0x392d16c666fb526b77db1e14f2769e23b06ec209badf92ce737f19734622203d</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -874,22 +866,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>75.19</t>
+          <t>109.09</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2175</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -914,7 +906,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xa0f6617255819010f00be4fb75d4597b30a12ae0fb712dd0c531651c52923088</t>
+          <t>0xca0eca2f3775c1a08e62703b0bc5096c0190a2a3e31600680143794ea7df898c</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786893336</t>
+          <t>1786893337</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>345.701149</t>
+          <t>311.685714</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,12 +963,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x869c335bdd3d2636e2f37a4d6ae91ebd65feaf4d359d1dbc8a5638d0d44406d8</t>
+          <t>0xd0bd4ac629ca0911ce51fad27d2f6e4e238bbaa1d989cbe664817ee4ebfcb2fc</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,29 +978,29 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>283.08</t>
+          <t>75.19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5375</t>
+          <t>1.2175</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>English Premier League</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Brentford 0</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>English Premier League</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>Brentford vs Tottenham Hotspur</t>
@@ -1026,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x116f827edbab2c40b76f0d489ef752efa0705d0d7281eb667522cfc3e453d283</t>
+          <t>0xa0f6617255819010f00be4fb75d4597b30a12ae0fb712dd0c531651c52923088</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1066,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>526.660465</t>
+          <t>345.701149</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,23 +1075,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x33233046e450a9042a0668b9a365ed1860e6833e33da55a35b5c6466d4648203</t>
+          <t>0x869c335bdd3d2636e2f37a4d6ae91ebd65feaf4d359d1dbc8a5638d0d44406d8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>29.60265</t>
+          <t>283.08</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.4825</t>
+          <t>1.5375</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1107,7 +1103,11 @@
           <t>English Premier League</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Brentford 0</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>English Premier League</t>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x5745247ce80bf8689dfe06022d99547fa927b160a694591736f58a9fb1d8b0b3</t>
+          <t>0x116f827edbab2c40b76f0d489ef752efa0705d0d7281eb667522cfc3e453d283</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>61.352642</t>
+          <t>526.660465</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x28b4cf2ef0b8471323b75e91b77f80e7f227ce9488635fc5dd9e23671ba1dcd4</t>
+          <t>0x33233046e450a9042a0668b9a365ed1860e6833e33da55a35b5c6466d4648203</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1195,81 +1195,73 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>29.60265</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.4825</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Brentford vs Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Brentford</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x5745247ce80bf8689dfe06022d99547fa927b160a694591736f58a9fb1d8b0b3</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19236538</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>221.34</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>1.45</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Over 3.0</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>English Premier League</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Brentford vs Tottenham Hotspur</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Brentford</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Tottenham Hotspur</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>0x3212fdea7fa0e385d3d02eb680e1ce50a1c7cb58afa9e7e34eb266a06ab18871</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>L19236538</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R8" t="inlineStr">
         <is>
           <t>1786893336</t>
@@ -1282,7 +1274,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>491.866667</t>
+          <t>61.352642</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x7d536b1f35b725269abc7254ec90ca50ccca56bb210b3d2118963062a41ce0b2</t>
+          <t>0x28b4cf2ef0b8471323b75e91b77f80e7f227ce9488635fc5dd9e23671ba1dcd4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1307,23 +1299,31 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>39.22095</t>
+          <t>221.34</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.315</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>English Premier League</t>
@@ -1331,27 +1331,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Hull City vs Manchester United</t>
+          <t>Brentford vs Tottenham Hotspur</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Hull City</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Manchester United</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x2cf719d8125a0ce8b30cf64e54c5ecf77f06126bc554e7b25fabbc72ee413952</t>
+          <t>0x3212fdea7fa0e385d3d02eb680e1ce50a1c7cb58afa9e7e34eb266a06ab18871</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19236539</t>
+          <t>L19236538</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1376,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786884152</t>
+          <t>1786893336</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1787398200</t>
+          <t>1787416200</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>124.510952</t>
+          <t>491.866667</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,28 +1403,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x3b4020a7dedef04108fd84d51b986ec0aa64b0e777c9ac0d4c51f107d3590106</t>
+          <t>0x7d536b1f35b725269abc7254ec90ca50ccca56bb210b3d2118963062a41ce0b2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>6.47</t>
+          <t>39.22095</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.2138</t>
+          <t>1.315</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xff94b64540b1f4876a9b61f7abc856bf1efeb99bca7cf7fc56e51fbe432c69a3</t>
+          <t>0x2cf719d8125a0ce8b30cf64e54c5ecf77f06126bc554e7b25fabbc72ee413952</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786880633</t>
+          <t>1786884152</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>30.269006</t>
+          <t>124.510952</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,28 +1507,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xe4c2b9f486982b41626561d2f921b54a2cc40bdf036a0442449bf08b0d587a84</t>
+          <t>0x3b4020a7dedef04108fd84d51b986ec0aa64b0e777c9ac0d4c51f107d3590106</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>123.26515</t>
+          <t>6.47</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5787</t>
+          <t>1.2138</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0xfa50abbae5bfdbf97cd2a58fbf350d5eba025159d6ca11f20066807fbf6cfcd2</t>
+          <t>0xff94b64540b1f4876a9b61f7abc856bf1efeb99bca7cf7fc56e51fbe432c69a3</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786880266</t>
+          <t>1786880633</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>212.98514</t>
+          <t>30.269006</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1611,7 +1611,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x0353c141478d0566f83e374f7784af6eb93f5721a343bd2253347a401c09996e</t>
+          <t>0xe4c2b9f486982b41626561d2f921b54a2cc40bdf036a0442449bf08b0d587a84</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1622,17 +1622,17 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>60.54972</t>
+          <t>123.26515</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.6738</t>
+          <t>1.5787</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1658,55 +1658,159 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
+          <t>0xfa50abbae5bfdbf97cd2a58fbf350d5eba025159d6ca11f20066807fbf6cfcd2</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19236539</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1786880266</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1787398200</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>212.98514</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0x0353c141478d0566f83e374f7784af6eb93f5721a343bd2253347a401c09996e</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>60.54972</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.6738</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>English Premier League</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Hull City vs Manchester United</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>0x0a08e0170f01c3d1a9a1ac32f64197e2b46643bdbadcccc75996936c0470d731</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>L19236539</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>1786880265</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>1787398200</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>89.869714</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>